<commit_message>
Correct partner belief to $52k vs real ~$59k buildout list
Co-authored-by: cesarblendss-ai <cesarblendss-ai@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/finance/buildout-cesar-reconciliation.xlsx
+++ b/finance/buildout-cesar-reconciliation.xlsx
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -515,10 +515,11 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Yellow = your stated numbers. Partner thinks ~$42k total — your list adds higher. Paper $29,835 is close to HALF of the full list sum (see below).</t>
-        </is>
-      </c>
-    </row>
+          <t>Yellow = your stated numbers. Partner thinks ~$52k total — your list is ~$58.8k (closer to $60k). Paper $29,835 ≈ half of the real total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -700,6 +701,7 @@
         <v>15985.25</v>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -829,10 +831,11 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>PARTNER “thinks we spent $42k”</t>
+          <t>PARTNER “thinks we spent $52k”</t>
         </is>
       </c>
     </row>
@@ -860,7 +863,7 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>42000</v>
+        <v>52000</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
@@ -879,7 +882,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Higher than his 42k</t>
+          <t>Higher than his 52k</t>
         </is>
       </c>
     </row>
@@ -890,7 +893,7 @@
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>16841</v>
+        <v>6841</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
@@ -916,11 +919,11 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>25% of HIS $42k belief</t>
+          <t>25% of HIS $52k belief</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>10500</v>
+        <v>13000</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
@@ -958,6 +961,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
@@ -1060,6 +1064,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
@@ -1070,14 +1075,47 @@
     <row r="46" ht="100" customHeight="1">
       <c r="A46" s="12" t="inlineStr">
         <is>
-          <t>Your list adds to $58,841.00 — that is the shop cost from these lines, not $42k and not $29,835.
-$29,835 on paper is almost exactly half of that list ($29,420.50) — gap only $414.50.
-Contractor is $13,800 split 50/50 → $6,900 each.
-Partner undercounting: his $42k vs your list $58,841.00 = he is missing ~$16,841.00.
-Still unknown / to find: anything beyond this list (other cards, Venmo, pre-Jan, furniture cash, etc.).</t>
-        </is>
-      </c>
-    </row>
+          <t>Your list adds to $58,841.00 (~$59k, basically the $60k capital story).
+Partner thinks $52,000 — he is short by ~$6,841.
+Your paper $29,835 ≈ half of the real pile (half of $58,841 = $29,420.50).
+Contractor $13,800 split 50/50 → $6,900 each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:E2"/>

</xml_diff>